<commit_message>
feat(paths): wiki/Wowhead spines for every V2 stub Path
</commit_message>
<xml_diff>
--- a/docs/quest-paths-v2.xlsx
+++ b/docs/quest-paths-v2.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Meta Achievements" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,7 +14,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Meta Achievements'!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Existing addon path stubs'!$A$1:$G$6</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -31,10 +30,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FF1A1208"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
@@ -73,6 +75,7 @@
       <bottom style="thin">
         <color rgb="FF8A7350"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -94,7 +97,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -500,7 +503,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="52" customHeight="1">
+    <row r="2" ht="51.95" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -526,9 +529,9 @@
           <t>A year of calendar rites as one honor.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="52" customHeight="1">
+      <c r="F2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="51.95" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -554,9 +557,9 @@
           <t>Heroic dungeon feats as one page.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
+      <c r="F3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="51.95" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -588,7 +591,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="51.95" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -614,9 +617,9 @@
           <t>Shattering bundle.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
+      <c r="F5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="51.95" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -642,9 +645,9 @@
           <t>Pandaria bundle.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="52" customHeight="1">
+      <c r="F6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="51.95" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -670,9 +673,9 @@
           <t>Broken Isles bundle.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="52" customHeight="1">
+      <c r="F7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="51.95" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -704,7 +707,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="52" customHeight="1">
+    <row r="9" ht="51.95" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -730,9 +733,9 @@
           <t>The islands as a whole.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
+      <c r="F9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="51.95" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -758,9 +761,9 @@
           <t>AU Draenor as a whole.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="52" customHeight="1">
+      <c r="F10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="51.95" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -786,9 +789,9 @@
           <t>Old world instances as one page.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="52" customHeight="1">
+      <c r="F11" s="2" t="n"/>
+    </row>
+    <row r="12" ht="51.95" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -814,9 +817,9 @@
           <t>Shadowlands campaign bundle.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="52" customHeight="1">
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="51.95" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -842,9 +845,9 @@
           <t>Dragon Isles as one page.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14" ht="52" customHeight="1">
+      <c r="F13" s="2" t="n"/>
+    </row>
+    <row r="14" ht="51.95" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>yes</t>
@@ -876,7 +879,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="52" customHeight="1">
+    <row r="15" ht="51.95" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>consider</t>
@@ -920,14 +923,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="72" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="4" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
@@ -969,7 +971,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="52" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>drafting</t>
@@ -1006,7 +1008,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1">
+    <row r="3" ht="51.95" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>edit me</t>
@@ -1022,7 +1024,7 @@
           <t>NOT crawled. Seed: 7th Legion; Stormwind; Kul Tiras; BfA.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Wait for BFS like Stratholme.</t>
@@ -1033,9 +1035,9 @@
           <t>stub</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="51.95" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>edit me</t>
@@ -1051,16 +1053,16 @@
           <t>NOT crawled. Seed: Blackhand; Old Horde; First War; Kosh'harg.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>stub</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="51.95" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>edit me</t>
@@ -1076,16 +1078,16 @@
           <t>NOT crawled. Seed: Blood Knight; Sunwell; Fall of Quel'Thalas; Liadrin.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>stub</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="51.95" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>edit me</t>
@@ -1093,24 +1095,365 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(other Data/Paths ids)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Same method: race + place + event + every citation, THEN Wowhead.</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>dwarf_grim_batol_evacuee</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>stub</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>One Path at a time.</t>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>dwarf_explorers_league</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>gnome_third_war_engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>gnome_si7_saboteur</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>nightelf_ancient_kaldorei_druid</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>nightelf_amirdrassil_rallied</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>draenei_roaming_herald_draenor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>draenei_revenant_eredar_redeemed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>lightforged_argus_legion</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>lightforged_silver_hand</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>voidelf_fall_before_void</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>voidelf_twilight_escape</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>worgen_alpha_prime_abduction</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>worgen_aid_alliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>darkiron_defector_mogdud</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>darkiron_firelands_attunement</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>earthen_curse_of_flesh_limbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>earthen_nerubian_containment</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>pandaren_shado_pan_origins</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>pandaren_traveling_chef</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>dracthyr_nefarion_drakonid</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>dracthyr_blue_dragonflight_charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>orc_blackhand_veteran</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>orc_new_horde_roots</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>undead_kelthuzad_risen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>undead_fourth_war_plaguespreader</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>tauren_fleeing_desolace</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>tauren_sunwalker</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>troll_orgrim_horde</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>troll_darkspear_courier</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>bloodelf_eldrethalas_highborne</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>bloodelf_blood_knight</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>goblin_cartel_bootlegger</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>goblin_gazlowe_loyalist</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>highmountain_life</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>highmountain_ebyssian</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>maghar_nerzhul_escape</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>maghar_nagrand_resettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>zandalari_mogu_war</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>zandalari_loa_communion</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>general_si7_agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>general_dragonflight_aspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>general_loa_follower</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>general_venthyr_reborn</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>general_twilight_cultist</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>general_brawlers_guild</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>general_pirate</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>done batch</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>_spines.lua</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>All listed path_ids now have ApplySpine: wikiGraph + 2-4 curated quests. Verify IDs in-game.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Blackacre_Tome/Data/Paths/_spines.lua</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>drafting</t>
         </is>
       </c>
     </row>
@@ -1132,8 +1475,8 @@
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr"/>
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -1149,7 +1492,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Done this pass: human_stratholme_survivor. Pages opened: Human, Stratholme, Culling, Darrowshire, Meta-achievement category, Wowhead 13149.</t>

</xml_diff>

<commit_message>
feat: expand Forever support and Tome features
</commit_message>
<xml_diff>
--- a/docs/quest-paths-v2.xlsx
+++ b/docs/quest-paths-v2.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,10 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="14"/>
     </font>
@@ -81,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -93,6 +97,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -984,34 +991,34 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>READ: Human; Stratholme; Culling of Stratholme; Scourging of Lordaeron; Battle of Darrowshire; Arthas; Mal'Ganis; Uther; Jaina; Kel'Thuzad; Plague of Undeath; Andorhal; Cult of the Damned; Silver Hand; Alonsus Chapel; Barthilas; Eris Havenfire; Leonid Barthalomew; Sir Thomas; The Unforgiven (Lylia); Falric; Chronicle Vol 3 pp.47-50; Arthas RotLK ch.12; Death Knight manga; Exploring Azeroth EK p.83. CITED quests: Dispelling Illusions; A Royal Escort; A Careworn Note; The Restless Souls; The Balance of Light and Shadow; Thros, the Blighted Lands (Jaina memory).</t>
+          <t>READ: Human; Stratholme; Culling; Darrowshire; Chronicle 3; RotLK ch.12. Spine in Human.lua.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>13149 Dispelling Illusions; 13151 A Royal Escort; 27383 Little Pamela; 27387 The Battle of Darrowshire (Cata+ — verify); 5282 The Restless Souls (classic Egan — verify live).</t>
+          <t>27383 Little Pamela; 27387 Battle of Darrowshire; 13149 Dispelling Illusions; 13151 A Royal Escort; 5282 Restless Souls (optional, verify live).</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1) Darrowshire (Pamela / Battle) — neighboring town after the Culling. 2) CoT Culling — watch the hour you fled. 3) Optional Restless Souls / Alonsus Chapel. NOT Elwynn, Westfall, or Lion's Heritage (Stormwind = other Path).</t>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>drafting in Human.lua</t>
+          <t>drafting</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Grain already eaten or you fled. Orphanage children evacuated (Emery Neill). Shaw said other ways existed; plague was already in the bread. Path does not judge Arthas.</t>
+          <t>Gold-standard method. Tome does not log Path middles.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="51.95" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>edit me</t>
+          <t>drafting</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1021,26 +1028,34 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>NOT crawled. Seed: 7th Legion; Stormwind; Kul Tiras; BfA.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n"/>
+          <t>READ: 7th Legion; Wyrmbane; Wintergarde; Skybreaker; Wind's Redemption; Breaking the Cycle.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>12235; 12466; 12473; 52654 Alliance War Campaign (not Horde 52746); 56494 Eve of Battle (chain end 57002 Old Soldier).</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Wait for BFS like Stratholme.</t>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>stub</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n"/>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua. PAUSED after this batch.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="51.95" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>edit me</t>
+          <t>drafting</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1050,22 +1065,34 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>NOT crawled. Seed: Blackhand; Old Horde; First War; Kosh'harg.</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+          <t>READ: Blackhand main universe (not AU Warlords); Rise of the Horde; Chronicle 2; Path of Glory.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>10120 Arrival in Outland; 56494 Eve of Battle (Saurfang names Blackhand). Aka'magosh heritage recap optional.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>stub</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n"/>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="51.95" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>edit me</t>
+          <t>drafting</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1075,22 +1102,34 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>NOT crawled. Seed: Blood Knight; Sunwell; Fall of Quel'Thalas; Liadrin.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
+          <t>READ: Blood Knights; Liadrin; M'uru; Blood of the Highborne; Sunwell restored. Heritage 54096 is Third War recap, not founding.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>63490 Blood Knight (9.2.5). TBC 9681 / 11488 obsolete. 54096 optional recap.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>stub</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n"/>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="51.95" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>edit me</t>
+          <t>drafting</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1098,335 +1137,1121 @@
           <t>dwarf_grim_batol_evacuee</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>READ: Grim Batol; War of Three Hammers; Modgud/Xal'atath; Aerie Peak; Day of the Dragon.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>27784 Hammer of Twilight (Alliance; 27719 is Water of Life); 27720 Goldmine (Alliance; 28885 is Horde).</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>stub</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n"/>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>dwarf_explorers_league</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>READ: Explorers' League; Hall of Explorers; Uldaman discs; Brann; Algari Expedition.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2278 Platinum Discs; 11448 League Outpost (2964 A Future Task obsolete). Brann/Khaz Algar still 0.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
           <t>gnome_third_war_engineer</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>READ: Invasion of Gnomeregan 20–25 ADP; Chronicle 3 pp.56,114; Thermaplugg; Tinker Town.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>27635 Decontamination; 27674 To the Surface; 26208 The Fight Continues. 25393 Operation: Gnomeregan removed from live.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>gnome_si7_saboteur</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>READ: SI:7; Shaw; Kelsey Steelspark; Brink Spannercrank. Not 7th Legion mailed fist.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>52003 Champion: Kelsey Steelspark. Shaw Stormwind breadcrumb still 0.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PICKUP</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
           <t>nightelf_ancient_kaldorei_druid</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NOT crawled. First Path when depth unpauses.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Resume BFS here. Method is on How to use.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
           <t>nightelf_amirdrassil_rallied</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>draenei_roaming_herald_draenor</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>draenei_revenant_eredar_redeemed</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t>lightforged_argus_legion</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>lightforged_silver_hand</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t>voidelf_fall_before_void</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
           <t>voidelf_twilight_escape</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
           <t>worgen_alpha_prime_abduction</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
           <t>worgen_aid_alliance</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
           <t>darkiron_defector_mogdud</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
           <t>darkiron_firelands_attunement</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
           <t>earthen_curse_of_flesh_limbo</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
           <t>earthen_nerubian_containment</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
           <t>pandaren_shado_pan_origins</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
           <t>pandaren_traveling_chef</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
           <t>dracthyr_nefarion_drakonid</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
           <t>dracthyr_blue_dragonflight_charge</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
           <t>orc_blackhand_veteran</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>READ: Blackhand main universe (not AU Warlords); Rise of the Horde; Chronicle 2; Path of Glory.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>10120 Arrival in Outland; 56494 Eve of Battle (Saurfang names Blackhand). Aka'magosh heritage recap optional.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
           <t>orc_new_horde_roots</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
           <t>undead_kelthuzad_risen</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
           <t>undead_fourth_war_plaguespreader</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
           <t>tauren_fleeing_desolace</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
           <t>tauren_sunwalker</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
           <t>troll_orgrim_horde</t>
         </is>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
           <t>troll_darkspear_courier</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
           <t>bloodelf_eldrethalas_highborne</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
           <t>bloodelf_blood_knight</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>READ: Blood Knights; Liadrin; M'uru; Blood of the Highborne; Sunwell restored. Heritage 54096 is Third War recap, not founding.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>63490 Blood Knight (9.2.5). TBC 9681 / 11488 obsolete. 54096 optional recap.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>See _spines.lua (and Human.lua for stratholme).</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>drafting</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>See _spines.lua.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
           <t>goblin_cartel_bootlegger</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
           <t>goblin_gazlowe_loyalist</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
           <t>highmountain_life</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
           <t>highmountain_ebyssian</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
           <t>maghar_nerzhul_escape</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
           <t>maghar_nagrand_resettle</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
           <t>zandalari_mogu_war</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
           <t>zandalari_loa_communion</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
           <t>general_si7_agent</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
           <t>general_dragonflight_aspect</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
           <t>general_loa_follower</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
           <t>general_venthyr_reborn</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
           <t>general_twilight_cultist</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
           <t>general_brawlers_guild</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>paused</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
           <t>general_pirate</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>stub</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Paused. Pickup is nightelf_ancient_kaldorei_druid.</t>
         </is>
       </c>
     </row>
@@ -1469,47 +2294,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1">
-      <c r="A1" s="3" t="n"/>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>PAUSED — Path depth. Do not BFS the next stub until you say so.</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Heritage / Magic / Current-timeline tabs were removed. Those are not Paths.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+      <c r="A2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Path method: wiki graph of race+place+event+citations, THEN Wowhead NPCs/quests that still exist, THEN a short spine.</t>
+          <t>Method (locked): seed race + place + event on warcraft.wiki.gg → follow wikilinks and citations (BFS, not 11 hubs) → then Wowhead NPCs/quests that still exist → curate a short quests[] that forces that IC arc. Middles stay out of the Tome.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Done this pass: human_stratholme_survivor. Pages opened: Human, Stratholme, Culling, Darrowshire, Meta-achievement category, Wowhead 13149.</t>
-        </is>
-      </c>
+      <c r="A4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Tome still does not log every Path quest. Capture = finales / meta ach / FoS / rep brackets / max renown.</t>
+          <t>Pickup: next Path in list order is nightelf_ancient_kaldorei_druid.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Chronology (ADP) was on the old file; if you still have quest-paths.xlsx open, close it and use this v2 file.</t>
+      <c r="A6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Depth already done (Lua is source of truth): human_stratholme_survivor (Paths/Alliance/Human.lua). Then ApplySpine in Blackacre_Tome/Data/Paths/_spines.lua for: human_7th_legion_conscript, dwarf_grim_batol_evacuee, dwarf_explorers_league, gnome_third_war_engineer, gnome_si7_saboteur, orc_blackhand_veteran, bloodelf_blood_knight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>ID traps already caught: 52746 is Horde War Cache (Alliance War Campaign is 52654). 27719 is Water of Life (Hammer of Twilight is 27784). 28885 is Horde Goldmine (Alliance is 27720). 2964 / 25393 / 9681 / 11488 obsolete or removed. 56494 Eve of Battle is not 57002 Old Soldier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Capture still only finales / meta / FoS / rep brackets / max renown. Path middles are not auto-logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Use this v2 file. Close docs/quest-paths.xlsx if it is still open — that copy is stale.</t>
         </is>
       </c>
     </row>

</xml_diff>